<commit_message>
test: pruebas unitarias con pytest (41 ejecuciones) e informe de pruebas con su sección
- tests/test_unitarias.py: reglas de negocio probadas de forma aislada (stubs de la
  sesión, de la orden y de la consulta SQL), con valores límite y particiones.
- Informe de pruebas: nueva sección 5 (unidad, quién/cómo/cuándo, driver pytest vs
  JUnit/TestNG, ejemplos, resultados por unidad, criterio de liberación).
- Documentos y README: 267 pruebas (226 de integración/funcionales + 41 unitarias).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/entrega-2do-corte/01_Plan_de_gestion_del_proyecto/Puntos_de_Funcion_y_PERT_StockPot.xlsx
+++ b/docs/entrega-2do-corte/01_Plan_de_gestion_del_proyecto/Puntos_de_Funcion_y_PERT_StockPot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\stockpot\docs\entrega-2do-corte\01_Plan_de_gestion_del_proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D86866F-D9DB-47D1-84B8-2124E98A8C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E380103-D3C2-4DC1-9804-9F9EE8D0CFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1044" yWindow="1440" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2136,7 +2136,7 @@
         <v>17</v>
       </c>
       <c r="I5" s="27">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -2223,7 +2223,7 @@
         <v>17</v>
       </c>
       <c r="I8" s="27">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -2484,7 +2484,7 @@
         <v>17</v>
       </c>
       <c r="I17" s="27">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
@@ -2629,7 +2629,7 @@
         <v>17</v>
       </c>
       <c r="I22" s="27">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
@@ -2658,7 +2658,7 @@
         <v>17</v>
       </c>
       <c r="I23" s="27">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
@@ -2745,7 +2745,7 @@
         <v>17</v>
       </c>
       <c r="I26" s="27">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
@@ -2890,7 +2890,7 @@
         <v>17</v>
       </c>
       <c r="I31" s="27">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
@@ -3818,7 +3818,7 @@
         <v>17</v>
       </c>
       <c r="I63" s="27">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
@@ -3905,7 +3905,7 @@
         <v>17</v>
       </c>
       <c r="I66" s="27">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
@@ -3934,7 +3934,7 @@
         <v>17</v>
       </c>
       <c r="I67" s="27">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
@@ -3992,7 +3992,7 @@
         <v>17</v>
       </c>
       <c r="I69" s="27">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
@@ -4195,7 +4195,7 @@
         <v>17</v>
       </c>
       <c r="I76" s="27">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
@@ -4311,7 +4311,7 @@
         <v>17</v>
       </c>
       <c r="I80" s="27">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>